<commit_message>
Fix bufomorph attack flip via masked layering and document open-mouth authoring.
Gameplay uses BiteAttack with faithful hip motion on Bufomorph_; enable upper-body split at Bufomorph_ Spine so locomotion keeps the hips planted. Add pose/motion diagnostics, IdleLookAround jaw validation, and defect evidence for pack-faithful open mouth.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -5727,6 +5727,11 @@
           <t>Death</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Bufomorph_ Spine</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>

<commit_message>
Independent import-pipeline review: locate Bufomorph 100x translation and lost reference pose; withdraw split-bone workaround; add runtime identity diagnostics and glTF-level merge prototype.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -5727,11 +5727,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Bufomorph_ Spine</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>

<commit_message>
Implement Option B pilot export for Bufomorph and Muscomorph on agent-c.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -2105,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.85546875" bestFit="1" customWidth="1" style="36" min="1" max="1"/>
@@ -3666,6 +3666,58 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>weapon_bufomorph_primary</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bufomorph Attack</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>BiteAttack</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3677,7 +3729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3982,7 +4034,6 @@
           <t>GetHit</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>CrawlLeft</t>
@@ -4039,7 +4090,6 @@
           <t>GetHit1</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>CrawlLeft</t>
@@ -4068,8 +4118,6 @@
           <t>IdleBreathe</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>3.5</v>
       </c>
@@ -4083,12 +4131,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4124,8 +4166,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>TurnLeft</t>
@@ -4177,12 +4217,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4218,8 +4252,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>CrawlLeft</t>
@@ -4248,8 +4280,6 @@
           <t>Idle</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>3.5</v>
       </c>
@@ -4258,13 +4288,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4300,12 +4323,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4341,8 +4358,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>CrawlLeft</t>
@@ -4399,11 +4414,6 @@
           <t>GetHit</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4439,12 +4449,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4480,12 +4484,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4521,12 +4519,6 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4562,12 +4554,47 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>bufomorph</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IdleLookAround</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>GetHitFront</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15851,7 +15878,50 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>U-0029</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bufomorph</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bufomorph</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>assets\units\bufomorph.glb</t>
+        </is>
+      </c>
       <c r="P21" s="11" t="n"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>bufomorph</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>weapon_bufomorph_primary</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="22">
       <c r="P22" s="11" t="n"/>
@@ -15888,7 +15958,6 @@
       <c r="O28" s="10" t="n"/>
       <c r="P28" s="12" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30" ht="15.75" customHeight="1" s="36">
       <c r="A30" s="7" t="inlineStr">
         <is>

</xml_diff>